<commit_message>
#6 C2 Change In BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Oil-Diffuser-A-v1.0.0/BOM/eSpark-BOM-Oil-Diffuser-A-v1.0.0.xlsx
+++ b/Design Files/Oil-Diffuser-A-v1.0.0/BOM/eSpark-BOM-Oil-Diffuser-A-v1.0.0.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="212">
   <si>
     <t>Component list</t>
   </si>
@@ -645,6 +645,18 @@
   </si>
   <si>
     <t>24V0.5A New AC 100V-240V Converter Switching Power Adapter DC 24V 0.5A 500mA Universla Power Supply EU Plug Tablet Charger</t>
+  </si>
+  <si>
+    <t>±10% 50V 100nF X7R Plugin,P=2.54mm Multilayer Ceramic Capacitors MLCC - Leaded ROHS</t>
+  </si>
+  <si>
+    <t>178MU0006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KNSCHA </t>
+  </si>
+  <si>
+    <t>C5632430</t>
   </si>
 </sst>
 </file>
@@ -1906,7 +1918,7 @@
       </c>
       <c r="Q8" s="14"/>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" ht="48">
       <c r="A9" s="1"/>
       <c r="B9" s="17">
         <f t="shared" ref="B9:B29" si="0">ROW(B9) - ROW($B$7)</f>
@@ -1919,22 +1931,22 @@
         <v>24</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>48</v>
+        <v>208</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>198</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>72</v>
+        <v>209</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>106</v>
+        <v>210</v>
       </c>
       <c r="I9" s="50" t="s">
         <v>199</v>
       </c>
       <c r="J9" s="20" t="s">
-        <v>125</v>
+        <v>211</v>
       </c>
       <c r="K9" s="20" t="s">
         <v>145</v>
@@ -1943,17 +1955,17 @@
         <v>1</v>
       </c>
       <c r="M9" s="14">
-        <v>2</v>
-      </c>
-      <c r="N9" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="N9" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="O9" s="21" t="s">
-        <v>176</v>
+      <c r="O9" s="21">
+        <v>1.1900000000000001E-2</v>
       </c>
       <c r="P9" s="21">
         <f t="shared" ref="P9" si="1">O9*M9</f>
-        <v>1.2847999999999999</v>
+        <v>0.59500000000000008</v>
       </c>
       <c r="Q9" s="20"/>
     </row>
@@ -3203,7 +3215,7 @@
       <c r="O34" s="54"/>
       <c r="P34" s="18">
         <f>SUM(P8:P33)</f>
-        <v>29.5473</v>
+        <v>28.857500000000002</v>
       </c>
       <c r="Q34" s="1"/>
     </row>
@@ -3233,11 +3245,11 @@
     <hyperlink ref="N12" r:id="rId18"/>
     <hyperlink ref="N11" r:id="rId19"/>
     <hyperlink ref="N10" r:id="rId20"/>
-    <hyperlink ref="N9" r:id="rId21"/>
-    <hyperlink ref="N8" r:id="rId22"/>
-    <hyperlink ref="N31" r:id="rId23"/>
-    <hyperlink ref="N32" r:id="rId24"/>
-    <hyperlink ref="N33" r:id="rId25"/>
+    <hyperlink ref="N8" r:id="rId21"/>
+    <hyperlink ref="N31" r:id="rId22"/>
+    <hyperlink ref="N32" r:id="rId23"/>
+    <hyperlink ref="N33" r:id="rId24"/>
+    <hyperlink ref="N9" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId26"/>

</xml_diff>